<commit_message>
2026-09-21 run: add operator-confirmed photos for SN 863 and 864
Operator confirmed which uploads belong to serials the OCR could not
read on its own:
  PCMRS0700863 → IMG_1486, IMG_1488
  PCMRS0700864 → IMG_1490, IMG_1492

Applied as manual overrides in the OCR cache and re-ran the match +
xlsx build. Coverage 5/8 → 7/8.

PCMRS0700883 still pending — IMG_1502-1504 (per operator) haven't been
uploaded to the OneDrive share yet; this run picks them up on the next
re-build once they land.
</commit_message>
<xml_diff>
--- a/shared/data/reshim-archive/2026-09-21/fargo_reshim_20260921_with_images.xlsx
+++ b/shared/data/reshim-archive/2026-09-21/fargo_reshim_20260921_with_images.xlsx
@@ -551,6 +551,216 @@
     <from>
       <col>15</col>
       <colOff>47625</colOff>
+      <row>5</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>16</col>
+      <colOff>-47625</colOff>
+      <row>6</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>16</col>
+      <colOff>47625</colOff>
+      <row>5</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>17</col>
+      <colOff>-47625</colOff>
+      <row>6</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>17</col>
+      <colOff>47625</colOff>
+      <row>5</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>18</col>
+      <colOff>-47625</colOff>
+      <row>6</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>15</col>
+      <colOff>47625</colOff>
+      <row>6</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>16</col>
+      <colOff>-47625</colOff>
+      <row>7</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>16</col>
+      <colOff>47625</colOff>
+      <row>6</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>17</col>
+      <colOff>-47625</colOff>
+      <row>7</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>17</col>
+      <colOff>47625</colOff>
+      <row>6</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>18</col>
+      <colOff>-47625</colOff>
+      <row>7</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>18</col>
+      <colOff>47625</colOff>
+      <row>6</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>19</col>
+      <colOff>-47625</colOff>
+      <row>7</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>15</col>
+      <colOff>47625</colOff>
       <row>8</row>
       <rowOff>47625</rowOff>
     </from>
@@ -562,11 +772,11 @@
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -592,11 +802,11 @@
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -622,11 +832,11 @@
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1373,10 +1583,18 @@
         </is>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" t="inlineStr"/>
-      <c r="O6" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>b4</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
@@ -1434,10 +1652,18 @@
         </is>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" t="inlineStr"/>
-      <c r="O7" t="inlineStr"/>
+        <v>4</v>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>b4</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
       <c r="P7" t="inlineStr"/>
       <c r="Q7" t="inlineStr"/>
       <c r="R7" t="inlineStr"/>
@@ -1587,7 +1813,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F25"/>
+  <dimension ref="A1:F23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1664,7 +1890,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10">
@@ -1674,7 +1900,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>18</v>
+        <v>11</v>
       </c>
     </row>
     <row r="11">
@@ -1840,34 +2066,10 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>PCMRS0700863</t>
+          <t>PCMRS0700883</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-09-19T01:39:06</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>PCMRS0700864</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>2026-09-19T00:37:14</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>PCMRS0700883</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
         <is>
           <t>2026-09-21T01:29:55</t>
         </is>

</xml_diff>

<commit_message>
2026-09-21 run: add operator-confirmed photos for SN 883
Final override for the day's flagged serial. Operator uploaded
IMG_1502-1504 after the previous rebuild; injecting them into the
OCR cache brings today's coverage to 8/8 with no gaps.
</commit_message>
<xml_diff>
--- a/shared/data/reshim-archive/2026-09-21/fargo_reshim_20260921_with_images.xlsx
+++ b/shared/data/reshim-archive/2026-09-21/fargo_reshim_20260921_with_images.xlsx
@@ -761,22 +761,112 @@
     <from>
       <col>15</col>
       <colOff>47625</colOff>
+      <row>7</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>16</col>
+      <colOff>-47625</colOff>
       <row>8</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
       <col>16</col>
+      <colOff>47625</colOff>
+      <row>7</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>17</col>
+      <colOff>-47625</colOff>
+      <row>8</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>17</col>
+      <colOff>47625</colOff>
+      <row>7</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>18</col>
+      <colOff>-47625</colOff>
+      <row>8</row>
+      <rowOff>-47625</rowOff>
+    </to>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </twoCellAnchor>
+  <twoCellAnchor editAs="oneCell">
+    <from>
+      <col>15</col>
+      <colOff>47625</colOff>
+      <row>8</row>
+      <rowOff>47625</rowOff>
+    </from>
+    <to>
+      <col>16</col>
       <colOff>-47625</colOff>
       <row>9</row>
       <rowOff>-47625</rowOff>
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId22"/>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -802,11 +892,11 @@
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId23"/>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -832,11 +922,11 @@
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId24"/>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1721,10 +1811,18 @@
         </is>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
-      </c>
-      <c r="N8" t="inlineStr"/>
-      <c r="O8" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>b4</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>OCR</t>
+        </is>
+      </c>
       <c r="P8" t="inlineStr"/>
       <c r="Q8" t="inlineStr"/>
       <c r="R8" t="inlineStr"/>
@@ -1813,7 +1911,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F23"/>
+  <dimension ref="A1:F22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1890,7 +1988,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="10">
@@ -2060,18 +2158,6 @@
       <c r="A22" t="inlineStr">
         <is>
           <t>SNs missing photos:</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>PCMRS0700883</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>2026-09-21T01:29:55</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
reshim archive: file 2026-09-19 as its own run, correct 2026-09-21
The published 2026-09-21 workbook held rows from three different plant
days. Against a live MES pull, SN 858 measures on 09-18 and 859-864 on
09-19; only 883 and 884 belong to 09-21, and 890-892 were missing
entirely. The row set looks photo-driven: the photo staging folder uses
a 48h lookback, so matching every OCR hit pulls neighbouring days in.

Both days are now regenerated by the pipeline against MES rather than
assembled from photos:

  2026-09-19  859-864          6 rows, 16 photos on 5 SNs
  2026-09-21  883,884,890-892  5 rows,  6 photos on 2 SNs

Regeneration reproduces the per-SN photo counts from the three earlier
"operator-confirmed photos" commits exactly, so no photo work is lost.
SN 858 and its 5 photos are not re-filed here; the archived 09-18 run
has its own discrepancy against MES and is left for a separate pass.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/shared/data/reshim-archive/2026-09-21/fargo_reshim_20260921_with_images.xlsx
+++ b/shared/data/reshim-archive/2026-09-21/fargo_reshim_20260921_with_images.xlsx
@@ -219,66 +219,6 @@
   </twoCellAnchor>
   <twoCellAnchor editAs="oneCell">
     <from>
-      <col>18</col>
-      <colOff>47625</colOff>
-      <row>1</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>19</col>
-      <colOff>-47625</colOff>
-      <row>2</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="4" name="Image 4" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId4"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>19</col>
-      <colOff>47625</colOff>
-      <row>1</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>20</col>
-      <colOff>-47625</colOff>
-      <row>2</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="5" name="Image 5" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId5"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
       <col>15</col>
       <colOff>47625</colOff>
       <row>2</row>
@@ -292,11 +232,11 @@
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="6" name="Image 6" descr="Picture"/>
+        <cNvPr id="4" name="Image 4" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId6"/>
+        <a:blip cstate="print" r:embed="rId4"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -322,11 +262,11 @@
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="7" name="Image 7" descr="Picture"/>
+        <cNvPr id="5" name="Image 5" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId7"/>
+        <a:blip cstate="print" r:embed="rId5"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -352,581 +292,11 @@
     </to>
     <pic>
       <nvPicPr>
-        <cNvPr id="8" name="Image 8" descr="Picture"/>
+        <cNvPr id="6" name="Image 6" descr="Picture"/>
         <cNvPicPr/>
       </nvPicPr>
       <blipFill>
-        <a:blip cstate="print" r:embed="rId8"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>47625</colOff>
-      <row>3</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>-47625</colOff>
-      <row>4</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="9" name="Image 9" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId9"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>47625</colOff>
-      <row>3</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>-47625</colOff>
-      <row>4</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="10" name="Image 10" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId10"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>17</col>
-      <colOff>47625</colOff>
-      <row>3</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>-47625</colOff>
-      <row>4</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="11" name="Image 11" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId11"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>47625</colOff>
-      <row>4</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>-47625</colOff>
-      <row>5</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="12" name="Image 12" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId12"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>47625</colOff>
-      <row>4</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>-47625</colOff>
-      <row>5</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="13" name="Image 13" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId13"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>17</col>
-      <colOff>47625</colOff>
-      <row>4</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>-47625</colOff>
-      <row>5</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="14" name="Image 14" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId14"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>47625</colOff>
-      <row>5</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>-47625</colOff>
-      <row>6</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="15" name="Image 15" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId15"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>47625</colOff>
-      <row>5</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>-47625</colOff>
-      <row>6</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="16" name="Image 16" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId16"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>17</col>
-      <colOff>47625</colOff>
-      <row>5</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>-47625</colOff>
-      <row>6</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="17" name="Image 17" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId17"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>47625</colOff>
-      <row>6</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>-47625</colOff>
-      <row>7</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="18" name="Image 18" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId18"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>47625</colOff>
-      <row>6</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>-47625</colOff>
-      <row>7</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="19" name="Image 19" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId19"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>17</col>
-      <colOff>47625</colOff>
-      <row>6</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>-47625</colOff>
-      <row>7</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="20" name="Image 20" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId20"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>18</col>
-      <colOff>47625</colOff>
-      <row>6</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>19</col>
-      <colOff>-47625</colOff>
-      <row>7</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="21" name="Image 21" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId21"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>47625</colOff>
-      <row>7</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>-47625</colOff>
-      <row>8</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="22" name="Image 22" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId22"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>47625</colOff>
-      <row>7</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>-47625</colOff>
-      <row>8</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="23" name="Image 23" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId23"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>17</col>
-      <colOff>47625</colOff>
-      <row>7</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>-47625</colOff>
-      <row>8</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="24" name="Image 24" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId24"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>15</col>
-      <colOff>47625</colOff>
-      <row>8</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>16</col>
-      <colOff>-47625</colOff>
-      <row>9</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="25" name="Image 25" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId25"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>16</col>
-      <colOff>47625</colOff>
-      <row>8</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>17</col>
-      <colOff>-47625</colOff>
-      <row>9</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="26" name="Image 26" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId26"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </blipFill>
-      <spPr>
-        <a:prstGeom prst="rect"/>
-      </spPr>
-    </pic>
-    <clientData/>
-  </twoCellAnchor>
-  <twoCellAnchor editAs="oneCell">
-    <from>
-      <col>17</col>
-      <colOff>47625</colOff>
-      <row>8</row>
-      <rowOff>47625</rowOff>
-    </from>
-    <to>
-      <col>18</col>
-      <colOff>-47625</colOff>
-      <row>9</row>
-      <rowOff>-47625</rowOff>
-    </to>
-    <pic>
-      <nvPicPr>
-        <cNvPr id="27" name="Image 27" descr="Picture"/>
-        <cNvPicPr/>
-      </nvPicPr>
-      <blipFill>
-        <a:blip cstate="print" r:embed="rId27"/>
+        <a:blip cstate="print" r:embed="rId6"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -1229,7 +599,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U9"/>
+  <dimension ref="A1:U6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="16" max="16"/>
@@ -1350,12 +720,12 @@
     <row r="2" ht="157.5" customHeight="1">
       <c r="A2" t="inlineStr">
         <is>
-          <t>PCMRS0700858</t>
+          <t>PCMRS0700883</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>X900.QTF.902.A01</t>
+          <t>X900.QTR.902.A01</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1364,16 +734,16 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.7</v>
+        <v>1.039999961853027</v>
       </c>
       <c r="E2" t="n">
-        <v>0.72</v>
+        <v>0.8100000023841858</v>
       </c>
       <c r="F2" t="n">
-        <v>1.32</v>
+        <v>1.039999961853027</v>
       </c>
       <c r="G2" t="n">
-        <v>0.46</v>
+        <v>0.4300000071525574</v>
       </c>
       <c r="H2" t="n">
         <v>0.35</v>
@@ -1393,11 +763,11 @@
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>2026-09-18T03:08:12</t>
+          <t>2026-09-21T11:57:00.033000</t>
         </is>
       </c>
       <c r="M2" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="N2" t="inlineStr">
         <is>
@@ -1419,12 +789,12 @@
     <row r="3" ht="157.5" customHeight="1">
       <c r="A3" t="inlineStr">
         <is>
-          <t>PCMRS0700859</t>
+          <t>PCMRS0700884</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>X900.QTF.902.A01</t>
+          <t>X900.QTR.902.A01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1433,16 +803,16 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>1.08</v>
+        <v>1.139999985694885</v>
       </c>
       <c r="E3" t="n">
-        <v>0.64</v>
+        <v>0.7400000095367432</v>
       </c>
       <c r="F3" t="n">
-        <v>1.4</v>
+        <v>0.9900000095367432</v>
       </c>
       <c r="G3" t="n">
-        <v>0.42</v>
+        <v>0.449999988079071</v>
       </c>
       <c r="H3" t="n">
         <v>0.35</v>
@@ -1462,7 +832,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>2026-09-18T10:19:54</t>
+          <t>2026-09-21T07:12:24.833000</t>
         </is>
       </c>
       <c r="M3" t="n">
@@ -1488,12 +858,12 @@
     <row r="4" ht="157.5" customHeight="1">
       <c r="A4" t="inlineStr">
         <is>
-          <t>PCMRS0700860</t>
+          <t>PCMRS0700890</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>X900.QTF.902.A01</t>
+          <t>X900.RTF.902.A01</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1502,16 +872,16 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1.1</v>
+        <v>1.110000014305115</v>
       </c>
       <c r="E4" t="n">
-        <v>0.79</v>
+        <v>0.6700000166893005</v>
       </c>
       <c r="F4" t="n">
-        <v>1.05</v>
+        <v>2.029999971389771</v>
       </c>
       <c r="G4" t="n">
-        <v>0.36</v>
+        <v>0.3700000047683716</v>
       </c>
       <c r="H4" t="n">
         <v>0.35</v>
@@ -1531,22 +901,14 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>2026-09-19T02:32:56</t>
+          <t>2026-09-21T12:11:16.410000</t>
         </is>
       </c>
       <c r="M4" t="n">
-        <v>3</v>
-      </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>b4</t>
-        </is>
-      </c>
-      <c r="O4" t="inlineStr">
-        <is>
-          <t>OCR</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N4" t="inlineStr"/>
+      <c r="O4" t="inlineStr"/>
       <c r="P4" t="inlineStr"/>
       <c r="Q4" t="inlineStr"/>
       <c r="R4" t="inlineStr"/>
@@ -1557,12 +919,12 @@
     <row r="5" ht="157.5" customHeight="1">
       <c r="A5" t="inlineStr">
         <is>
-          <t>PCMRS0700862</t>
+          <t>PCMRS0700891</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>X900.QTF.902.A01</t>
+          <t>X900.RTF.902.A01</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1571,16 +933,16 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>1.06</v>
+        <v>1.179999947547913</v>
       </c>
       <c r="E5" t="n">
-        <v>0.76</v>
+        <v>0.8999999761581421</v>
       </c>
       <c r="F5" t="n">
-        <v>1</v>
+        <v>1.549999952316284</v>
       </c>
       <c r="G5" t="n">
-        <v>0.37</v>
+        <v>0.3700000047683716</v>
       </c>
       <c r="H5" t="n">
         <v>0.35</v>
@@ -1600,22 +962,14 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>2026-09-19T01:38:49</t>
+          <t>2026-09-21T16:46:49.700000</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>3</v>
-      </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>b4</t>
-        </is>
-      </c>
-      <c r="O5" t="inlineStr">
-        <is>
-          <t>OCR</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N5" t="inlineStr"/>
+      <c r="O5" t="inlineStr"/>
       <c r="P5" t="inlineStr"/>
       <c r="Q5" t="inlineStr"/>
       <c r="R5" t="inlineStr"/>
@@ -1626,12 +980,12 @@
     <row r="6" ht="157.5" customHeight="1">
       <c r="A6" t="inlineStr">
         <is>
-          <t>PCMRS0700863</t>
+          <t>PCMRS0700892</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>X900.QTF.902.A01</t>
+          <t>X900.RTF.902.A01</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1640,16 +994,16 @@
         </is>
       </c>
       <c r="D6" t="n">
-        <v>1.14</v>
+        <v>0.8600000143051147</v>
       </c>
       <c r="E6" t="n">
-        <v>0.77</v>
+        <v>0.7799999713897705</v>
       </c>
       <c r="F6" t="n">
-        <v>1.02</v>
+        <v>1.870000004768372</v>
       </c>
       <c r="G6" t="n">
-        <v>0.42</v>
+        <v>0.449999988079071</v>
       </c>
       <c r="H6" t="n">
         <v>0.35</v>
@@ -1669,235 +1023,20 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>2026-09-19T01:39:06</t>
+          <t>2026-09-21T16:25:08.880000</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>3</v>
-      </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>b4</t>
-        </is>
-      </c>
-      <c r="O6" t="inlineStr">
-        <is>
-          <t>OCR</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="N6" t="inlineStr"/>
+      <c r="O6" t="inlineStr"/>
       <c r="P6" t="inlineStr"/>
       <c r="Q6" t="inlineStr"/>
       <c r="R6" t="inlineStr"/>
       <c r="S6" t="inlineStr"/>
       <c r="T6" t="inlineStr"/>
       <c r="U6" t="inlineStr"/>
-    </row>
-    <row r="7" ht="157.5" customHeight="1">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>PCMRS0700864</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>X900.QTF.902.A01</t>
-        </is>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="D7" t="n">
-        <v>1.09</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0.82</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1.08</v>
-      </c>
-      <c r="G7" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="H7" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="J7" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="K7" t="inlineStr">
-        <is>
-          <t>1_&lt;0.5</t>
-        </is>
-      </c>
-      <c r="L7" t="inlineStr">
-        <is>
-          <t>2026-09-19T00:37:14</t>
-        </is>
-      </c>
-      <c r="M7" t="n">
-        <v>4</v>
-      </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>b4</t>
-        </is>
-      </c>
-      <c r="O7" t="inlineStr">
-        <is>
-          <t>OCR</t>
-        </is>
-      </c>
-      <c r="P7" t="inlineStr"/>
-      <c r="Q7" t="inlineStr"/>
-      <c r="R7" t="inlineStr"/>
-      <c r="S7" t="inlineStr"/>
-      <c r="T7" t="inlineStr"/>
-      <c r="U7" t="inlineStr"/>
-    </row>
-    <row r="8" ht="157.5" customHeight="1">
-      <c r="A8" t="inlineStr">
-        <is>
-          <t>PCMRS0700883</t>
-        </is>
-      </c>
-      <c r="B8" t="inlineStr">
-        <is>
-          <t>X900.QTR.902.A01</t>
-        </is>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="D8" t="n">
-        <v>0.98</v>
-      </c>
-      <c r="E8" t="n">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="F8" t="n">
-        <v>1.04</v>
-      </c>
-      <c r="G8" t="n">
-        <v>0.43</v>
-      </c>
-      <c r="H8" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="I8" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="J8" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="K8" t="inlineStr">
-        <is>
-          <t>1_&lt;0.5</t>
-        </is>
-      </c>
-      <c r="L8" t="inlineStr">
-        <is>
-          <t>2026-09-21T01:29:55</t>
-        </is>
-      </c>
-      <c r="M8" t="n">
-        <v>3</v>
-      </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>b4</t>
-        </is>
-      </c>
-      <c r="O8" t="inlineStr">
-        <is>
-          <t>OCR</t>
-        </is>
-      </c>
-      <c r="P8" t="inlineStr"/>
-      <c r="Q8" t="inlineStr"/>
-      <c r="R8" t="inlineStr"/>
-      <c r="S8" t="inlineStr"/>
-      <c r="T8" t="inlineStr"/>
-      <c r="U8" t="inlineStr"/>
-    </row>
-    <row r="9" ht="157.5" customHeight="1">
-      <c r="A9" t="inlineStr">
-        <is>
-          <t>PCMRS0700884</t>
-        </is>
-      </c>
-      <c r="B9" t="inlineStr">
-        <is>
-          <t>X900.QTR.902.A01</t>
-        </is>
-      </c>
-      <c r="C9" t="inlineStr">
-        <is>
-          <t>600</t>
-        </is>
-      </c>
-      <c r="D9" t="n">
-        <v>1.14</v>
-      </c>
-      <c r="E9" t="n">
-        <v>0.74</v>
-      </c>
-      <c r="F9" t="n">
-        <v>0.99</v>
-      </c>
-      <c r="G9" t="n">
-        <v>0.45</v>
-      </c>
-      <c r="H9" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="I9" t="n">
-        <v>0.46</v>
-      </c>
-      <c r="J9" t="inlineStr">
-        <is>
-          <t>OK</t>
-        </is>
-      </c>
-      <c r="K9" t="inlineStr">
-        <is>
-          <t>1_&lt;0.5</t>
-        </is>
-      </c>
-      <c r="L9" t="inlineStr">
-        <is>
-          <t>2026-09-21T01:12:45</t>
-        </is>
-      </c>
-      <c r="M9" t="n">
-        <v>3</v>
-      </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>b4</t>
-        </is>
-      </c>
-      <c r="O9" t="inlineStr">
-        <is>
-          <t>OCR</t>
-        </is>
-      </c>
-      <c r="P9" t="inlineStr"/>
-      <c r="Q9" t="inlineStr"/>
-      <c r="R9" t="inlineStr"/>
-      <c r="S9" t="inlineStr"/>
-      <c r="T9" t="inlineStr"/>
-      <c r="U9" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1911,7 +1050,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F22"/>
+  <dimension ref="A1:F25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1928,7 +1067,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -1948,7 +1087,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -1988,7 +1127,7 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="10">
@@ -1998,7 +1137,7 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>11</v>
+        <v>24</v>
       </c>
     </row>
     <row r="11">
@@ -2008,7 +1147,7 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="13">
@@ -2050,10 +1189,10 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="C14" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="D14" t="n">
         <v>0</v>
@@ -2102,14 +1241,14 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>X900.QTF.902.A01</t>
+          <t>X900.QTR.902.A01</t>
         </is>
       </c>
       <c r="B17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="C17" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D17" t="n">
         <v>0</v>
@@ -2126,14 +1265,14 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>X900.QTR.902.A01</t>
+          <t>X900.RTF.902.A01</t>
         </is>
       </c>
       <c r="B18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D18" t="n">
         <v>0</v>
@@ -2158,6 +1297,42 @@
       <c r="A22" t="inlineStr">
         <is>
           <t>SNs missing photos:</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>PCMRS0700890</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>2026-09-21T12:11:16.410000</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>PCMRS0700891</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>2026-09-21T16:46:49.700000</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>PCMRS0700892</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>2026-09-21T16:25:08.880000</t>
         </is>
       </c>
     </row>

</xml_diff>